<commit_message>
Add 22 more Horimiya grammar patterns and dedupe re-pasted rows.
Duplicate detection now also matches timestamp plus example sentence, so reworded versions of existing lines keep the original entry.
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -818,6 +818,490 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>57s</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>If you knew [過去形/事実]</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>...if you knew how much I love...</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>（もし）〜だと知っていたら</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1:04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>[主語] thought that would [動詞]</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>He thought that would cheer me up.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>[主語]はそれが[動詞]すると思った</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1:04</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>cheer [人] up</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>...cheer me up.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>[人]を元気づける</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1:08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>What goes on in [人]'s head?</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Just what goes on in his head?</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>[人]の頭の中はどうなってるの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1:12</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ask [人] for [モノ/事]</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>...asking me for your phone number...</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>[人]に[モノ/事]を求める</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1:18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>have the guts to [動詞]</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>He didn't have the guts to ask...</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>[動詞]する度胸がある</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1:24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Who's up for [名詞/動名詞]?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Yo, who's up for some bad singing?</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>[名詞/動名詞]したい人？</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1:30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>What a steal!</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Half off, two hours. What a steal.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>激安だ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1:35</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>I think I'm gonna pass.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Ah, I think I'm gonna pass.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>（今回は）やめておくよ</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1:56</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>[人/モノ] sounded so [形容詞]</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Oh, he sounded so depressed.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>[人/モノ]がとても[形容詞]に聞こえた</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1:59</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Then again...</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Then again, that's kind of his thing.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>そうは言っても</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1:59</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>That's kind of [人]'s thing.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>...that's kind of his thing.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>それは[人]のいつものやつだ</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2:07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>[主語] has to be [名詞/形容詞]</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>He has to be.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>[主語]は絶対に[名詞/形容詞]だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2:12</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>pick up [モノ/事]</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Does your nerd alert pick up anything?</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>[モノ/事]を感知する</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2:18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>I don't even know if [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>I don't even know if Miyamura has...</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>[主語が〜する]かどうかすら分からない</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2:20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>gotta [動詞]</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Gotta run.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>[動詞]しなきゃ</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>It feels like [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>It feels like she hurries home every day.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>[主語が〜している]気がする</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2:28</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>[名詞] or something</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Must be a boyfriend or something.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>[名詞]か何か</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2:31</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>way [形容詞]</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Well, she's way popular.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>めちゃくちゃ[形容詞]だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2:54</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Got it.</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Got it.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>了解</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2:55</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>I'll handle [モノ/事]</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>I'll handle dinner.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>[モノ/事]は私が処理するよ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2:57</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>[モノ/事] sucks.</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Overtime sucks, I know.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>[モノ/事]は最悪だ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace the first 17 Horimiya patterns with the revised wording.
Placeholders are now generalized (subject and object slots instead of fixed pronouns) and the Japanese glosses are shortened to one reading each.
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -452,7 +452,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>That's all for [today / now]</t>
+          <t>That's all for [名詞]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[ today / now ] はこれで終わり / 以上だ</t>
+          <t>[名詞]はこれで以上だ</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[モノ/事] will eat up my time</t>
+          <t>[主語] will eat up [モノ/事]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -484,7 +484,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>[モノ/事]が時間を食いつぶす・費やす</t>
+          <t>[主語]が[モノ/事]を食いつぶす</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>most of my [名詞]</t>
+          <t>most of [名詞]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[名詞]の大半 / ほとんど</t>
+          <t>[名詞]の大半</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[人]に[動詞]するよう促す / 勧める</t>
+          <t>[人]に[動詞]するよう勧める</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>while you still can</t>
+          <t>while [主語+動詞]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>（あなたが）できるうちに / できる間は</t>
+          <t>[主語]が[動詞]できるうちに</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>喜んで[動詞]しますよ / （もし〜なら）〜したいところです</t>
+          <t>喜んで[動詞]する</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Why would you [動詞]?</t>
+          <t>Why would [主語] [動詞]?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>なんで（あなたが）[動詞]なんてするの？ / なぜ〜するわけ？</t>
+          <t>なんで[主語]が[動詞]なんてするの？</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>（[人]に）ついて行く / 同行する</t>
+          <t>（[人]に）ついて行く</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>[形容詞]な態度をとるな / 〜にするな</t>
+          <t>[形容詞]な態度をとるな</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>[モノ/事]が関わっている / 絡んでいる</t>
+          <t>[モノ/事]が関わっているとき</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>大人の監視 / 監督が必要だ</t>
+          <t>大人の監視が必要だ</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>（それは）理にかなっている / 納得だ / 確かにそうだね</t>
+          <t>それは理にかなっている</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[行動/発言] is baffling</t>
+          <t>[主語] is baffling</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>[行動/発言]が理解不能だ / 呆れ果てる</t>
+          <t>[主語]が理解不能だ</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>お墨付きの[名詞] / 誰もが認める[名詞]</t>
+          <t>誰もが認める[名詞]</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>馬鹿なこと / くだらないこと</t>
+          <t>くだらないこと</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>元気を出して / うつむかないで</t>
+          <t>元気を出して</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 22 Horimiya patterns from the 3:03-5:59 range.
Duplicate detection now compares the English skeleton as well, so two patterns taught from one example sentence both survive while reworded repeats are still dropped.
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>while [主語+動詞]</t>
+          <t>while [主語] still can</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[主語]が[動詞]できるうちに</t>
+          <t>[主語]ができるうちに</t>
         </is>
       </c>
     </row>
@@ -1299,6 +1299,490 @@
       <c r="D40" t="inlineStr">
         <is>
           <t>[モノ/事]は最悪だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>3:03</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>should probably get going</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>I should probably get going.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>そろそろ行かなくちゃ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>3:07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>have been [動詞ing]</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>We've been waiting for you.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ずっと[動詞]し続けている</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>3:07</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>wait for [人/モノ]</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>We've been waiting for you.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>[人/モノ]を待つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>3:16</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>hit up [場所/人]</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Let's hit up that store...</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>[場所/人]に行く・連絡する</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>3:16</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>while [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>...while we're here.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>[主語]が[動詞]している間に</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>3:19</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Why not?</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Why not?</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>いいじゃない</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>5:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>on [人]'s day off</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>...working on her day off.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>[人]の休日に</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>5:03</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>too [形容詞] for [人]'s own good</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>...she's too nice for her own good.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>[形容詞]すぎて本人のためにならない</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>5:07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>I wish [主語] would [動詞]</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>I wish she'd learn how to...</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>[主語]が[動詞]してくれたらいいのに</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>5:07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>say [言葉] to [人]</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>...how to say no to people.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>[人]に[言葉]を言う</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>5:18</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>[モノ/事] happen to [人]</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>...what happened to your little nose?</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>[人]に[モノ/事]が起こる</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>5:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>fall down</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>I fell down.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>転ぶ</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>5:29</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>have / get [モノ/事] taken care of</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>...since you've got it taken care of.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>[モノ/事]を片付けてもらう</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>5:34</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>cause [人] trouble</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Hope he didn't cause you too much trouble.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>[人]に迷惑をかける</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>5:45</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>be in a hurry</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>...if you're not in any sort of hurry...</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>急いでいる</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>5:45</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>any sort of [名詞]</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>...if you're not in any sort of hurry...</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>何らかの[名詞]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>5:48</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>more than [形容詞]</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>...you're more than welcome to stay...</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>十分に[形容詞]だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>5:48</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>for a while</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>...to stay for a while.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>しばらくの間</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>5:52</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>[人]'s way of [動名詞ing]</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>This will be my way of saying thanks.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>[人]なりの[動詞]する方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>5:56</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>[主語] spook [人]</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>...because this dog spooked him.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>[主語]が[人]を驚かせる</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>5:59</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>I appreciate [人] [動名詞ing]</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>I appreciate you helping him out.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>[人]が[動詞]してくれて感謝する</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>5:59</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>help [人] out</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>...helping him out.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>[人]を助ける</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 16 Horimiya patterns from the 6:01-6:52 range.
Placeholder notation matches the existing gerund slots and each gloss keeps a single reading.
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1786,6 +1786,358 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>6:01</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>appreciate [人] for [名詞/動名詞]</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>...I appreciate you for treating me.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>[人]の[名詞/動名詞]に感謝する</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>6:03</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Why do you [動詞] if [主語+動詞]?</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Why do you drink coffee if it tastes so gross?</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>[主語が〜]なら、なぜ[動詞]するの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>6:06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>ask myself the same thing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>I ask myself the same thing.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>自分でもそう思ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>6:09</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>introduce [自分]</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>He introduced himself...</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>自己紹介する</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>6:09</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>[言葉/行動] and everything</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>He introduced himself and everything.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>[言葉/行動]やら何やらすべて</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>6:12</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>That's nice of [人] to [動詞]</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>That's nice of you to say.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>[人]が[動詞]してくれて優しい</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>6:12</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>a real handful</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>He's a real handful...</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>本当に手に負えない</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>6:17</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>[主語] is what's really [形容詞]</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>...housework is what's really impressive.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>[主語]こそが本当に[形容詞]なことだ</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>6:21</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Never would have guessed.</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Never would have guessed, Hori.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>全く予想もつかなかった</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>6:28</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>How'd you know that?</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>...how'd you know that?</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>なんでそれ知ってるの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>6:32</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>the same [名詞] as [人/モノ]</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>...the same school as me?</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>[人/モノ]と同じ[名詞]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>6:36</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Are you being [形容詞] right now?</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Are you being serious right now?</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>今[形容詞]な態度をとってるの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>6:48</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>That can't be [人/モノ].</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>That can't be the same person.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>それが[人/モノ]なはずがない</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>6:50</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>[主語] doesn't make sense anymore</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>...the world doesn't make sense anymore.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>[主語]がもう意味をなさない</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>6:52</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>one of the [最上級] [複数名詞]</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>...one of the weirdest faces...</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>最も[形容詞]な[名詞]の一つ</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>6:52</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>in the history of [名詞]</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>...in the history of weird faces.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>[名詞]の歴史の中で</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 32 Horimiya patterns from the 7:07-8:54 range.
Splits the two senses of "pick up" into distinct slots so no English pattern maps to two different answers.
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D78"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>pick up [モノ/事]</t>
+          <t>pick up [信号/気配]</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>[モノ/事]を感知する</t>
+          <t>[信号/気配]を感知する</t>
         </is>
       </c>
     </row>
@@ -2135,6 +2135,710 @@
       <c r="D78" t="inlineStr">
         <is>
           <t>[名詞]の歴史の中で</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>7:07</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Got a sec?</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Miyamura, got a sec?</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ちょっと時間ある？</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>7:11</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>come over to [場所]</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>...come over to your house again?</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>[場所]へ遊びに来る</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>7:17</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>save [人] from [モノ/事]</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>...saved him from the dog...</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>[人]を[モノ/事]から救う</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>7:22</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>pick up [モノ]</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>I'll pick up a picture book...</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>[モノ]を買ってくる</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>7:24</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>[主語] will be enough</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>...showing up will be enough...</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>[主語]で十分だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>7:28</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>What a relief!</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>What a relief.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ホッとした</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>7:28</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>break [人]'s heart</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>...break Sota's heart.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>[人]をひどく傷つける</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>7:37</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>the fact that [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>By the fact that you sought me out...</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>[主語が〜する]という事実</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>7:37</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>seek [人] out</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>...you sought me out...</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>[人]を探し出す</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>7:39</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>after [過去の事/日] and all</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>...after yesterday and all.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>[過去の事/日]もあった後で</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>7:41</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>for sure</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>...I thought for sure you'd avoid me.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>間違いなく</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>7:44</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>that way</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>...react that way?</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>そんな風に</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>7:51</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>It freaks [人] out to [動詞]</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>It freaked me out to see...</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>[動詞]して[人]はびっくりする</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>7:51</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>a different side of [人]</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>...a different side of you...</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>[人]の意外な一面</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>7:54</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>out of [場所]</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>...out of school, too.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>[場所]の外で</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>7:56</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>a silly reason</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>...a pretty silly reason...</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>くだらない理由</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>7:56</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>straight up [動詞]</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>...to straight up avoid you.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>あからさまに[動詞]する</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>8:02</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>be not used to [動名詞/名詞]</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>I'm just not used to hearing...</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>[動名詞/名詞]に慣れていない</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>8:12</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>What's with [モノ/事]?</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>What's with the look?</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>[モノ/事]は一体どうしたの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>8:14</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>notice how [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>I just noticed how nice your smile is.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>[主語が〜であるか]に気づく</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>wear [髪] up</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>You should wear your hair up...</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>[髪]をアップにする</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>more often</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>...more often.</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>もっと頻繁に</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>lose [モノ]</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Maybe lose the glasses, too.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>[モノ]を外す</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>8:19</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Don't you think?</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Don't you think?</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>そう思わない？</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>8:24</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>quite a few</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>You do have quite a few.</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>かなりの数</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>8:24</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>What's the grand total?</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>So what's the grand total?</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>合計でいくつ（いくら）？</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>8:27</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>up to [数値]</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>It's up to nine.</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>最大で[数値]まで</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>8:27</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>along with [モノ/人]</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>...along with the one on my lip.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>[モノ/人]と一緒に</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>8:33</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>agree with [人]</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>My mom would agree with you.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>[人]に同意する</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>be into [モノ/事]</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>...I'm not into that moe nonsense.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>[モノ/事]にハマっている</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>8:51</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>like you wouldn't believe</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>...hurt like you wouldn't believe.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>信じられないほど（〜だ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>8:54</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>back in [過去の時期]</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>...back in middle school.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>[過去の時期]の頃に</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Horimiya patterns from 9:04 to 9:54
</commit_message>
<xml_diff>
--- a/data/horimiya.xlsx
+++ b/data/horimiya.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D110"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2842,6 +2842,270 @@
         </is>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>9:04</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>a straight-A [名詞]</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>...You're like a straight-A queen.</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>成績がオールAの[名詞]</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>9:09</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>What's incredible is [主語+動詞]</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>What's incredible is how a quiet guy...</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>驚きなのは[主語が〜する]ことだ</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>9:12</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Is that the rule?</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Is that the rule?</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>それがルールなの？</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>9:17</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>[人]'s initial impression of [人/モノ]</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>my initial impression of him</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>[人]が[人/モノ]に抱いた第一印象</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>9:18</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>couldn't have been further from [名詞/実態]</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>...couldn't have been further from the person...</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>[名詞/実態]とは全く違っていた</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>9:24</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>[モノ] is on sale</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Eggs are on sale tomorrow...</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>[モノ]がセール中だ</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>9:39</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>[事/モノ] lasts till [時間]</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>...only lasts till 4:00 p.m.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>[事/モノ]が[時間]まで続く</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>9:42</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>I've got this.</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>I mean, I've got this.</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>私に任せて</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>9:43</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>stand in [人]'s way</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Nothing's gonna stand in my way...</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>[人]の行く手を阻む</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>9:47</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>What are the odds?</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>But what are the odds?</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>まさかそんなことがあるなんて</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>9:51</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>report to [場所]</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>All committee members please report to...</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>[場所]に集合する</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>9:54</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>be called in for [名詞]</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>You're being called for an emergency meeting.</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>[名詞]のために呼び出される</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>